<commit_message>
Update data sources and scripts
</commit_message>
<xml_diff>
--- a/bof-web/public/data/settlement-sheet-new.xlsx
+++ b/bof-web/public/data/settlement-sheet-new.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -16,7 +16,7 @@
     <sheet name="Payroll" sheetId="1" r:id="rId1"/>
     <sheet name="Payroll Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -159,6 +159,9 @@
     <t>O. Lee</t>
   </si>
   <si>
+    <t>R. Johnson</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -217,9 +220,6 @@
   </si>
   <si>
     <t>Total Net Pay</t>
-  </si>
-  <si>
-    <t>R. Johnson</t>
   </si>
 </sst>
 </file>
@@ -229,9 +229,9 @@
   <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_-"/>
-    <numFmt numFmtId="179" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,13 +291,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -486,19 +486,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42422BCC-C81E-4C68-A409-0FDF30364344}">
   <dimension ref="A1:W13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
-    <col min="17" max="17" width="23.33203125" customWidth="1"/>
-    <col min="18" max="18" width="9.88671875" customWidth="1"/>
-    <col min="20" max="20" width="9.88671875" customWidth="1"/>
-    <col min="21" max="21" width="8.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="17" max="17" width="23.28515625" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" customWidth="1"/>
+    <col min="21" max="21" width="8.28515625" customWidth="1"/>
     <col min="22" max="22" width="17" customWidth="1"/>
     <col min="23" max="23" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -569,7 +569,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -650,7 +650,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -812,7 +812,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -974,7 +974,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -1460,9 +1460,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" s="8" customFormat="1">
       <c r="A13" s="4" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B13" s="4">
         <v>2230</v>
@@ -1580,161 +1580,161 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CF28E4B-1208-46B7-8CC7-1A8315458D6C}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <f>SUM(Payroll!B2:B13)</f>
         <v>25125</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="3">
         <f>SUM(Payroll!C2:C13)</f>
         <v>807</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <f>SUM(Payroll!D2:D13)</f>
         <v>25932</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5">
         <f>SUM(Payroll!E2:E13)</f>
         <v>1607.7839999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <f>SUM(Payroll!F2:F13)</f>
         <v>376.01400000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <f>SUM(Payroll!G2:G13)</f>
         <v>4667.76</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8">
         <f>SUM(Payroll!H2:H13)</f>
         <v>907.62000000000023</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B9">
         <f>SUM(Payroll!I2:I13)</f>
         <v>116.69399999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10">
         <f>SUM(Payroll!J2:J13)</f>
         <v>171.15120000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11">
         <f>SUM(Payroll!K2:K13)</f>
         <v>631.6</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12">
         <f>SUM(Payroll!L2:L13)</f>
         <v>361.89</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B13">
         <f>SUM(Payroll!M2:M13)</f>
         <v>272.10000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14">
         <f>SUM(Payroll!N2:N13)</f>
         <v>522.33000000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B15">
         <f>SUM(Payroll!O2:O13)</f>
         <v>304.52000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B16">
         <f>SUM(Payroll!P2:P13)</f>
         <v>455.81</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B17">
         <f>SUM(Payroll!Q2:Q13)</f>
         <v>14.280000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1743,18 +1743,18 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19">
         <f>SUM(Payroll!T2:T13)</f>
         <v>10409.553200000002</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B20">
         <f>SUM(Payroll!U2:U13)</f>

</xml_diff>